<commit_message>
Bridge private retail facts into daily close
</commit_message>
<xml_diff>
--- a/data/external_sources/retail_network_sales.xlsx
+++ b/data/external_sources/retail_network_sales.xlsx
@@ -5409,7 +5409,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:O25"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -5452,98 +5452,92 @@
         <v>Возвраты шт</v>
       </c>
       <c r="N1" t="str">
-        <v>Юр Лицо</v>
+        <v>1</v>
       </c>
       <c r="O1" t="str">
-        <v>Дата</v>
-      </c>
-      <c r="P1" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>Наименование</v>
+        <v>"Кровавый" пилинг для лица маркировки "Алтэя"</v>
       </c>
       <c r="B2" t="str">
-        <v>Номенклатура</v>
+        <v>99000076205</v>
       </c>
       <c r="C2" t="str">
-        <v>Артикул</v>
+        <v>krovavii_piling_30ml</v>
       </c>
       <c r="D2" t="str">
-        <v>Штрихкод</v>
+        <v>4670020498208</v>
       </c>
       <c r="E2" t="str">
-        <v>Заказано руб</v>
+        <v>8684</v>
       </c>
       <c r="F2" t="str">
-        <v>Доставлено руб</v>
+        <v>0</v>
       </c>
       <c r="G2" t="str">
-        <v>В пути руб</v>
+        <v>8684</v>
       </c>
       <c r="H2" t="str">
-        <v>Отменено руб</v>
+        <v>0</v>
       </c>
       <c r="I2" t="str">
-        <v>Заказано шт</v>
+        <v>13</v>
       </c>
       <c r="J2" t="str">
-        <v>Доставлено шт</v>
+        <v>0</v>
       </c>
       <c r="K2" t="str">
-        <v>В пути шт</v>
+        <v>13</v>
       </c>
       <c r="L2" t="str">
-        <v>Отменено шт</v>
+        <v>0</v>
       </c>
       <c r="M2" t="str">
-        <v>Возвраты шт</v>
+        <v>0</v>
       </c>
       <c r="N2" t="str">
         <v>1</v>
       </c>
       <c r="O2" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P2" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Крем для лица с ретинолом 0.5, сыворотка от морщин и пигментных пятен, Алтея, Ретидерм, 50 мл</v>
+        <v>Гель для проблемной кожи лица и тела, с маркировками Алтея</v>
       </c>
       <c r="B3" t="str">
-        <v>99000076216</v>
+        <v>99000114730</v>
       </c>
       <c r="C3" t="str">
-        <v>retiderm_50ml</v>
+        <v>gel_antiakne_20ml_v2</v>
       </c>
       <c r="D3" t="str">
-        <v>4.61017E+12</v>
+        <v>4660417420110</v>
       </c>
       <c r="E3" t="str">
-        <v>11918</v>
+        <v>7928</v>
       </c>
       <c r="F3" t="str">
         <v>0</v>
       </c>
       <c r="G3" t="str">
-        <v>11918</v>
+        <v>7928</v>
       </c>
       <c r="H3" t="str">
         <v>0</v>
       </c>
       <c r="I3" t="str">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="J3" t="str">
         <v>0</v>
       </c>
       <c r="K3" t="str">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="L3" t="str">
         <v>0</v>
@@ -5555,48 +5549,45 @@
         <v>1</v>
       </c>
       <c r="O3" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P3" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>"Кровавый" пилинг для лица маркировки "Алтэя"</v>
+        <v>Продукция косметическая для ухода за кожей, в том числе в наборах: Маска для проблемной кожи лица м</v>
       </c>
       <c r="B4" t="str">
-        <v>99000076205</v>
+        <v>99000114727</v>
       </c>
       <c r="C4" t="str">
-        <v>krovavii_piling_30ml</v>
+        <v>maska_dlya_lica_100m</v>
       </c>
       <c r="D4" t="str">
-        <v>4.67002E+12</v>
+        <v>4670020498741</v>
       </c>
       <c r="E4" t="str">
-        <v>10181</v>
+        <v>6213</v>
       </c>
       <c r="F4" t="str">
-        <v>584</v>
+        <v>0</v>
       </c>
       <c r="G4" t="str">
-        <v>9597</v>
+        <v>5274</v>
       </c>
       <c r="H4" t="str">
-        <v>0</v>
+        <v>939</v>
       </c>
       <c r="I4" t="str">
-        <v>18</v>
+        <v>7</v>
       </c>
       <c r="J4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" t="str">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="L4" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" t="str">
         <v>0</v>
@@ -5605,45 +5596,42 @@
         <v>1</v>
       </c>
       <c r="O4" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P4" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Гель для проблемной кожи лица и тела, с маркировками Алтея</v>
+        <v>Крем для лица с ретинолом 0.5, сыворотка от морщин и пигментных пятен, Алтея, Ретидерм, 50 мл</v>
       </c>
       <c r="B5" t="str">
-        <v>99000114730</v>
+        <v>99000076216</v>
       </c>
       <c r="C5" t="str">
-        <v>gel_antiakne_20ml_v2</v>
+        <v>retiderm_50ml</v>
       </c>
       <c r="D5" t="str">
-        <v>4.66042E+12</v>
+        <v>4610172186219</v>
       </c>
       <c r="E5" t="str">
-        <v>9842</v>
+        <v>5944</v>
       </c>
       <c r="F5" t="str">
-        <v>0</v>
+        <v>498</v>
       </c>
       <c r="G5" t="str">
-        <v>9842</v>
+        <v>5446</v>
       </c>
       <c r="H5" t="str">
         <v>0</v>
       </c>
       <c r="I5" t="str">
-        <v>17</v>
+        <v>25</v>
       </c>
       <c r="J5" t="str">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K5" t="str">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="L5" t="str">
         <v>0</v>
@@ -5655,45 +5643,42 @@
         <v>1</v>
       </c>
       <c r="O5" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P5" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Крем c ретинолом для век антивозрастной для кожи и кожи вокруг глаз, 30мл</v>
+        <v>Крем для волос Упругий завиток, 300 мл</v>
       </c>
       <c r="B6" t="str">
-        <v>99000154005</v>
+        <v>99000114726</v>
       </c>
       <c r="C6" t="str">
-        <v>retinol_boost_krem_d</v>
+        <v>curly_method_300ml</v>
       </c>
       <c r="D6" t="str">
-        <v>4.66042E+12</v>
+        <v>4603320465441</v>
       </c>
       <c r="E6" t="str">
-        <v>8297</v>
+        <v>5815</v>
       </c>
       <c r="F6" t="str">
         <v>0</v>
       </c>
       <c r="G6" t="str">
-        <v>8297</v>
+        <v>5815</v>
       </c>
       <c r="H6" t="str">
         <v>0</v>
       </c>
       <c r="I6" t="str">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J6" t="str">
         <v>0</v>
       </c>
       <c r="K6" t="str">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="L6" t="str">
         <v>0</v>
@@ -5705,33 +5690,30 @@
         <v>1</v>
       </c>
       <c r="O6" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P6" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Крем для волос Упругий завиток, 300 мл</v>
+        <v>Пенка для укладки волос</v>
       </c>
       <c r="B7" t="str">
-        <v>99000114726</v>
+        <v>99000125266</v>
       </c>
       <c r="C7" t="str">
-        <v>curly_method_300ml</v>
+        <v>penka_kudryavii_meto</v>
       </c>
       <c r="D7" t="str">
-        <v>4.60332E+12</v>
+        <v>4670020498611</v>
       </c>
       <c r="E7" t="str">
-        <v>6195</v>
+        <v>4831</v>
       </c>
       <c r="F7" t="str">
         <v>0</v>
       </c>
       <c r="G7" t="str">
-        <v>6195</v>
+        <v>4831</v>
       </c>
       <c r="H7" t="str">
         <v>0</v>
@@ -5755,48 +5737,45 @@
         <v>1</v>
       </c>
       <c r="O7" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P7" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>РЕТИНАЙТ сыворотка для лица 30 мл</v>
+        <v>Крем-шелк для сухой кожи ног</v>
       </c>
       <c r="B8" t="str">
-        <v>99000125142</v>
+        <v>99000076225</v>
       </c>
       <c r="C8" t="str">
-        <v>retinait_syvorotka_1</v>
+        <v>kremshelk_100ml</v>
       </c>
       <c r="D8" t="str">
-        <v>4.60332E+12</v>
+        <v>4670020498437</v>
       </c>
       <c r="E8" t="str">
-        <v>5736</v>
+        <v>3776</v>
       </c>
       <c r="F8" t="str">
         <v>0</v>
       </c>
       <c r="G8" t="str">
-        <v>4096</v>
+        <v>3776</v>
       </c>
       <c r="H8" t="str">
-        <v>1640</v>
+        <v>0</v>
       </c>
       <c r="I8" t="str">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="J8" t="str">
         <v>0</v>
       </c>
       <c r="K8" t="str">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="L8" t="str">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M8" t="str">
         <v>0</v>
@@ -5805,10 +5784,7 @@
         <v>1</v>
       </c>
       <c r="O8" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P8" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="9">
@@ -5822,28 +5798,28 @@
         <v>retinait_krem_1_50ml</v>
       </c>
       <c r="D9" t="str">
-        <v>4.66042E+12</v>
+        <v>4660417421605</v>
       </c>
       <c r="E9" t="str">
-        <v>5116</v>
+        <v>3075</v>
       </c>
       <c r="F9" t="str">
-        <v>1025</v>
+        <v>0</v>
       </c>
       <c r="G9" t="str">
-        <v>4091</v>
+        <v>3075</v>
       </c>
       <c r="H9" t="str">
         <v>0</v>
       </c>
       <c r="I9" t="str">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J9" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K9" t="str">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="L9" t="str">
         <v>0</v>
@@ -5855,45 +5831,42 @@
         <v>1</v>
       </c>
       <c r="O9" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P9" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Пенка для укладки волос</v>
+        <v>Крем от растяжек, Алтея, 200 мл</v>
       </c>
       <c r="B10" t="str">
-        <v>99000125266</v>
+        <v>99000114731</v>
       </c>
       <c r="C10" t="str">
-        <v>penka_kudryavii_meto</v>
+        <v>krem_ot_rastyazhek</v>
       </c>
       <c r="D10" t="str">
-        <v>4.67002E+12</v>
+        <v>4670020497898</v>
       </c>
       <c r="E10" t="str">
-        <v>4759</v>
+        <v>2960</v>
       </c>
       <c r="F10" t="str">
         <v>0</v>
       </c>
       <c r="G10" t="str">
-        <v>4759</v>
+        <v>2960</v>
       </c>
       <c r="H10" t="str">
         <v>0</v>
       </c>
       <c r="I10" t="str">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" t="str">
         <v>0</v>
       </c>
       <c r="K10" t="str">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="L10" t="str">
         <v>0</v>
@@ -5905,33 +5878,30 @@
         <v>1</v>
       </c>
       <c r="O10" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P10" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Крем-шелк для сухой кожи ног</v>
+        <v>Спрей-сыворотка для волос маркировки Алтея</v>
       </c>
       <c r="B11" t="str">
-        <v>99000076225</v>
+        <v>99000076226</v>
       </c>
       <c r="C11" t="str">
-        <v>kremshelk_100ml</v>
+        <v>termo_sprei_200ml</v>
       </c>
       <c r="D11" t="str">
-        <v>4.67002E+12</v>
+        <v>4670020497980</v>
       </c>
       <c r="E11" t="str">
-        <v>3386</v>
+        <v>2614</v>
       </c>
       <c r="F11" t="str">
         <v>0</v>
       </c>
       <c r="G11" t="str">
-        <v>3386</v>
+        <v>2614</v>
       </c>
       <c r="H11" t="str">
         <v>0</v>
@@ -5955,10 +5925,7 @@
         <v>1</v>
       </c>
       <c r="O11" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P11" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="12">
@@ -5972,16 +5939,16 @@
         <v>spicul_gel_mask_75ml</v>
       </c>
       <c r="D12" t="str">
-        <v>4.66042E+12</v>
+        <v>4660417421858</v>
       </c>
       <c r="E12" t="str">
-        <v>3135</v>
+        <v>2523</v>
       </c>
       <c r="F12" t="str">
         <v>0</v>
       </c>
       <c r="G12" t="str">
-        <v>3135</v>
+        <v>2523</v>
       </c>
       <c r="H12" t="str">
         <v>0</v>
@@ -6005,45 +5972,42 @@
         <v>1</v>
       </c>
       <c r="O12" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P12" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея, 50 мл</v>
+        <v>Средство косметическое: Воск для волос торговой марки: «Алтея» 15гр</v>
       </c>
       <c r="B13" t="str">
-        <v>99000176496</v>
+        <v>99000131672</v>
       </c>
       <c r="C13" t="str">
-        <v>retinait_krem_1_5_50</v>
+        <v>vosk_stik_15ml</v>
       </c>
       <c r="D13" t="str">
-        <v>4.66042E+12</v>
+        <v>4670207150196</v>
       </c>
       <c r="E13" t="str">
-        <v>2319</v>
+        <v>2080</v>
       </c>
       <c r="F13" t="str">
         <v>0</v>
       </c>
       <c r="G13" t="str">
-        <v>2319</v>
+        <v>2080</v>
       </c>
       <c r="H13" t="str">
         <v>0</v>
       </c>
       <c r="I13" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J13" t="str">
         <v>0</v>
       </c>
       <c r="K13" t="str">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="L13" t="str">
         <v>0</v>
@@ -6055,45 +6019,42 @@
         <v>1</v>
       </c>
       <c r="O13" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P13" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Крем от растяжек, Алтея, 200 мл</v>
+        <v>Спрей для роста волос торговой марки Алтея</v>
       </c>
       <c r="B14" t="str">
-        <v>99000114731</v>
+        <v>99000114724</v>
       </c>
       <c r="C14" t="str">
-        <v>krem_ot_rastyazhek</v>
+        <v>sprei_buster_100ml</v>
       </c>
       <c r="D14" t="str">
-        <v>4.67002E+12</v>
+        <v>4603320465359</v>
       </c>
       <c r="E14" t="str">
-        <v>1728</v>
+        <v>1802</v>
       </c>
       <c r="F14" t="str">
         <v>0</v>
       </c>
       <c r="G14" t="str">
-        <v>1728</v>
+        <v>1802</v>
       </c>
       <c r="H14" t="str">
         <v>0</v>
       </c>
       <c r="I14" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J14" t="str">
         <v>0</v>
       </c>
       <c r="K14" t="str">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L14" t="str">
         <v>0</v>
@@ -6105,45 +6066,42 @@
         <v>1</v>
       </c>
       <c r="O14" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P14" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Алтея Сыворотка для лица сыворотка для лица с ниацинамидом для лица антивозрастная, от пигментных пя</v>
+        <v>Ламеллярный крем для рук с мочевиной, увлажняющий и питательный с маслом кокоса, Алтея, 75 мл</v>
       </c>
       <c r="B15" t="str">
-        <v>99000182844</v>
+        <v>99000114729</v>
       </c>
       <c r="C15" t="str">
-        <v>syvorotka_dlya_lica_</v>
+        <v>krem_dlya_ruk_75ml</v>
       </c>
       <c r="D15" t="str">
-        <v>4.60331E+12</v>
+        <v>4660417421452</v>
       </c>
       <c r="E15" t="str">
-        <v>1698</v>
+        <v>1545</v>
       </c>
       <c r="F15" t="str">
         <v>0</v>
       </c>
       <c r="G15" t="str">
-        <v>1698</v>
+        <v>1545</v>
       </c>
       <c r="H15" t="str">
         <v>0</v>
       </c>
       <c r="I15" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J15" t="str">
         <v>0</v>
       </c>
       <c r="K15" t="str">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="L15" t="str">
         <v>0</v>
@@ -6155,45 +6113,42 @@
         <v>1</v>
       </c>
       <c r="O15" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P15" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Ретинайт 0,5 экспресс-омоложение Anti-Age Липосомальный комплекс ретинола 0,5 + Ниацинамид 50 мл</v>
+        <v>Крем c ретинолом для век антивозрастной для кожи и кожи вокруг глаз, 30мл</v>
       </c>
       <c r="B16" t="str">
-        <v>99000131675</v>
+        <v>99000154005</v>
       </c>
       <c r="C16" t="str">
-        <v>retinait_krem_05_50m</v>
+        <v>retinol_boost_krem_d</v>
       </c>
       <c r="D16" t="str">
-        <v>4.66042E+12</v>
+        <v>4660417421636</v>
       </c>
       <c r="E16" t="str">
-        <v>1289</v>
+        <v>893</v>
       </c>
       <c r="F16" t="str">
         <v>0</v>
       </c>
       <c r="G16" t="str">
-        <v>1289</v>
+        <v>893</v>
       </c>
       <c r="H16" t="str">
         <v>0</v>
       </c>
       <c r="I16" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J16" t="str">
         <v>0</v>
       </c>
       <c r="K16" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L16" t="str">
         <v>0</v>
@@ -6205,45 +6160,42 @@
         <v>1</v>
       </c>
       <c r="O16" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P16" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Спрей для роста волос торговой марки Алтея</v>
+        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея</v>
       </c>
       <c r="B17" t="str">
-        <v>99000114724</v>
+        <v>99000124418</v>
       </c>
       <c r="C17" t="str">
-        <v>sprei_buster_100ml</v>
+        <v>retinait_krem_025_50</v>
       </c>
       <c r="D17" t="str">
-        <v>4.60332E+12</v>
+        <v>4660417421599</v>
       </c>
       <c r="E17" t="str">
-        <v>1280</v>
+        <v>844</v>
       </c>
       <c r="F17" t="str">
         <v>0</v>
       </c>
       <c r="G17" t="str">
-        <v>1280</v>
+        <v>844</v>
       </c>
       <c r="H17" t="str">
         <v>0</v>
       </c>
       <c r="I17" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J17" t="str">
         <v>0</v>
       </c>
       <c r="K17" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L17" t="str">
         <v>0</v>
@@ -6255,42 +6207,39 @@
         <v>1</v>
       </c>
       <c r="O17" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P17" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Спрей-сыворотка для волос маркировки Алтея</v>
+        <v>Крем для лица spf 50 с защитой UVA/UVB, торговой марки Алтея</v>
       </c>
       <c r="B18" t="str">
-        <v>99000076226</v>
+        <v>99000163832</v>
       </c>
       <c r="C18" t="str">
-        <v>termo_sprei_200ml</v>
+        <v>krem_spf50_50ml</v>
       </c>
       <c r="D18" t="str">
-        <v>4.67002E+12</v>
+        <v>4660417421766</v>
       </c>
       <c r="E18" t="str">
-        <v>1220</v>
+        <v>800</v>
       </c>
       <c r="F18" t="str">
-        <v>616</v>
+        <v>0</v>
       </c>
       <c r="G18" t="str">
-        <v>604</v>
+        <v>800</v>
       </c>
       <c r="H18" t="str">
         <v>0</v>
       </c>
       <c r="I18" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J18" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K18" t="str">
         <v>1</v>
@@ -6305,33 +6254,30 @@
         <v>1</v>
       </c>
       <c r="O18" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P18" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Cыворотка SPICULBOOST торговой марки Алтея, 30 мл</v>
+        <v>Крем специального назначения «Псоридонт» 50 мл</v>
       </c>
       <c r="B19" t="str">
-        <v>99000179436</v>
+        <v>99000125141</v>
       </c>
       <c r="C19" t="str">
-        <v>spiculboost_30ml</v>
+        <v>psoral_50ml</v>
       </c>
       <c r="D19" t="str">
-        <v>4.63045E+12</v>
+        <v>4660417421087</v>
       </c>
       <c r="E19" t="str">
-        <v>1131</v>
+        <v>760</v>
       </c>
       <c r="F19" t="str">
         <v>0</v>
       </c>
       <c r="G19" t="str">
-        <v>1131</v>
+        <v>760</v>
       </c>
       <c r="H19" t="str">
         <v>0</v>
@@ -6355,45 +6301,42 @@
         <v>1</v>
       </c>
       <c r="O19" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P19" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Средство косметическое: Воск для волос торговой марки: «Алтея» 15гр</v>
+        <v>Ретинайт 0,5 экспресс-омоложение Anti-Age Липосомальный комплекс ретинола 0,5 + Ниацинамид 50 мл</v>
       </c>
       <c r="B20" t="str">
-        <v>99000131672</v>
+        <v>99000131675</v>
       </c>
       <c r="C20" t="str">
-        <v>vosk_stik_15ml</v>
+        <v>retinait_krem_05_50m</v>
       </c>
       <c r="D20" t="str">
-        <v>4.67021E+12</v>
+        <v>4660417421759</v>
       </c>
       <c r="E20" t="str">
-        <v>975</v>
+        <v>744</v>
       </c>
       <c r="F20" t="str">
         <v>0</v>
       </c>
       <c r="G20" t="str">
-        <v>975</v>
+        <v>744</v>
       </c>
       <c r="H20" t="str">
         <v>0</v>
       </c>
       <c r="I20" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J20" t="str">
         <v>0</v>
       </c>
       <c r="K20" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L20" t="str">
         <v>0</v>
@@ -6405,45 +6348,42 @@
         <v>1</v>
       </c>
       <c r="O20" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P20" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Ламеллярный крем для рук с мочевиной, увлажняющий и питательный с маслом кокоса, Алтея, 75 мл</v>
+        <v>Средство косметическое для ухода за волосами: маска для волос восстанавливающая с авокадо и маслом о</v>
       </c>
       <c r="B21" t="str">
-        <v>99000114729</v>
+        <v>99000076210</v>
       </c>
       <c r="C21" t="str">
-        <v>krem_dlya_ruk_75ml</v>
+        <v>maska-batter_250ml</v>
       </c>
       <c r="D21" t="str">
-        <v>4.66042E+12</v>
+        <v>4670020497546</v>
       </c>
       <c r="E21" t="str">
-        <v>928</v>
+        <v>657</v>
       </c>
       <c r="F21" t="str">
         <v>0</v>
       </c>
       <c r="G21" t="str">
-        <v>928</v>
+        <v>657</v>
       </c>
       <c r="H21" t="str">
         <v>0</v>
       </c>
       <c r="I21" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J21" t="str">
         <v>0</v>
       </c>
       <c r="K21" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L21" t="str">
         <v>0</v>
@@ -6455,33 +6395,30 @@
         <v>1</v>
       </c>
       <c r="O21" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P21" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Крем для век пробуждающий маркировки «Алтэя»</v>
+        <v>Средство косметическое профессиональное: маска разогревающая для роста волос торговой марки: Алтея.</v>
       </c>
       <c r="B22" t="str">
-        <v>99000125267</v>
+        <v>99000076208</v>
       </c>
       <c r="C22" t="str">
-        <v>krem_dlya_vek_30ml</v>
+        <v>maska-batter_dlya_ro</v>
       </c>
       <c r="D22" t="str">
-        <v>4.67002E+12</v>
+        <v>4603320465366</v>
       </c>
       <c r="E22" t="str">
-        <v>840</v>
+        <v>650</v>
       </c>
       <c r="F22" t="str">
         <v>0</v>
       </c>
       <c r="G22" t="str">
-        <v>840</v>
+        <v>650</v>
       </c>
       <c r="H22" t="str">
         <v>0</v>
@@ -6505,33 +6442,30 @@
         <v>1</v>
       </c>
       <c r="O22" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P22" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Средство косметическое для ухода за волосами: масло для бороды, маркировка: Алтея.</v>
+        <v>Шампунь от перхоти лечебный с климбазолом Алтея, 250мл</v>
       </c>
       <c r="B23" t="str">
-        <v>99000076215</v>
+        <v>99000076206</v>
       </c>
       <c r="C23" t="str">
-        <v>maslo_dlya_borodi_50</v>
+        <v>shampun_protiv_perho</v>
       </c>
       <c r="D23" t="str">
-        <v>4.61017E+12</v>
+        <v>4670020496679</v>
       </c>
       <c r="E23" t="str">
-        <v>718</v>
+        <v>650</v>
       </c>
       <c r="F23" t="str">
         <v>0</v>
       </c>
       <c r="G23" t="str">
-        <v>718</v>
+        <v>650</v>
       </c>
       <c r="H23" t="str">
         <v>0</v>
@@ -6555,33 +6489,30 @@
         <v>1</v>
       </c>
       <c r="O23" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P23" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Шампунь для роста волос, от выпадения волос профессиональный, Алтея, 250 мл</v>
+        <v>Средство косметическое для ухода за волосами: масло для бороды, маркировка: Алтея.</v>
       </c>
       <c r="B24" t="str">
-        <v>99000076213</v>
+        <v>99000076215</v>
       </c>
       <c r="C24" t="str">
-        <v>shampun_dlya_rosta_2</v>
+        <v>maslo_dlya_borodi_50</v>
       </c>
       <c r="D24" t="str">
-        <v>4.67002E+12</v>
+        <v>4610172186882</v>
       </c>
       <c r="E24" t="str">
-        <v>695</v>
+        <v>569</v>
       </c>
       <c r="F24" t="str">
         <v>0</v>
       </c>
       <c r="G24" t="str">
-        <v>695</v>
+        <v>569</v>
       </c>
       <c r="H24" t="str">
         <v>0</v>
@@ -6605,33 +6536,30 @@
         <v>1</v>
       </c>
       <c r="O24" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P24" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>Шампунь от перхоти лечебный с климбазолом Алтея, 250мл</v>
+        <v>Шампунь для роста волос, от выпадения волос профессиональный, Алтея, 250 мл</v>
       </c>
       <c r="B25" t="str">
-        <v>99000076206</v>
+        <v>99000076213</v>
       </c>
       <c r="C25" t="str">
-        <v>shampun_protiv_perho</v>
+        <v>shampun_dlya_rosta_2</v>
       </c>
       <c r="D25" t="str">
-        <v>4.67002E+12</v>
+        <v>4670020496747</v>
       </c>
       <c r="E25" t="str">
-        <v>680</v>
+        <v>461</v>
       </c>
       <c r="F25" t="str">
         <v>0</v>
       </c>
       <c r="G25" t="str">
-        <v>680</v>
+        <v>461</v>
       </c>
       <c r="H25" t="str">
         <v>0</v>
@@ -6655,172 +6583,19 @@
         <v>1</v>
       </c>
       <c r="O25" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P25" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="str">
-        <v>Сыворотка для лица с гиалуроновой кислотой маркировки "Алтэя"</v>
-      </c>
-      <c r="B26" t="str">
-        <v>99000076209</v>
-      </c>
-      <c r="C26" t="str">
-        <v>syvorotka_guk_30ml</v>
-      </c>
-      <c r="D26" t="str">
-        <v>4.67002E+12</v>
-      </c>
-      <c r="E26" t="str">
-        <v>671</v>
-      </c>
-      <c r="F26" t="str">
-        <v>0</v>
-      </c>
-      <c r="G26" t="str">
-        <v>671</v>
-      </c>
-      <c r="H26" t="str">
-        <v>0</v>
-      </c>
-      <c r="I26" t="str">
-        <v>1</v>
-      </c>
-      <c r="J26" t="str">
-        <v>0</v>
-      </c>
-      <c r="K26" t="str">
-        <v>1</v>
-      </c>
-      <c r="L26" t="str">
-        <v>0</v>
-      </c>
-      <c r="M26" t="str">
-        <v>0</v>
-      </c>
-      <c r="N26" t="str">
-        <v>1</v>
-      </c>
-      <c r="O26" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P26" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="str">
-        <v>Средства косметические для ухода за бровями: сыворотка для бровей и ресниц, с маркировкой "Алтея", 6</v>
-      </c>
-      <c r="B27" t="str">
-        <v>99000132524</v>
-      </c>
-      <c r="C27" t="str">
-        <v>syvorotka_dlya_rosta</v>
-      </c>
-      <c r="D27" t="str">
-        <v>4.65674E+12</v>
-      </c>
-      <c r="E27" t="str">
-        <v>488</v>
-      </c>
-      <c r="F27" t="str">
-        <v>0</v>
-      </c>
-      <c r="G27" t="str">
-        <v>488</v>
-      </c>
-      <c r="H27" t="str">
-        <v>0</v>
-      </c>
-      <c r="I27" t="str">
-        <v>1</v>
-      </c>
-      <c r="J27" t="str">
-        <v>0</v>
-      </c>
-      <c r="K27" t="str">
-        <v>1</v>
-      </c>
-      <c r="L27" t="str">
-        <v>0</v>
-      </c>
-      <c r="M27" t="str">
-        <v>0</v>
-      </c>
-      <c r="N27" t="str">
-        <v>1</v>
-      </c>
-      <c r="O27" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P27" t="str">
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="str">
-        <v>Гель для бровей с коллагеном и эластином, фиксация на 24 часа, Алтея, 5 мл</v>
-      </c>
-      <c r="B28" t="str">
-        <v>99000114725</v>
-      </c>
-      <c r="C28" t="str">
-        <v>gel_brows_5ml</v>
-      </c>
-      <c r="D28" t="str">
-        <v>4.67657E+12</v>
-      </c>
-      <c r="E28" t="str">
-        <v>400</v>
-      </c>
-      <c r="F28" t="str">
-        <v>0</v>
-      </c>
-      <c r="G28" t="str">
-        <v>400</v>
-      </c>
-      <c r="H28" t="str">
-        <v>0</v>
-      </c>
-      <c r="I28" t="str">
-        <v>1</v>
-      </c>
-      <c r="J28" t="str">
-        <v>0</v>
-      </c>
-      <c r="K28" t="str">
-        <v>1</v>
-      </c>
-      <c r="L28" t="str">
-        <v>0</v>
-      </c>
-      <c r="M28" t="str">
-        <v>0</v>
-      </c>
-      <c r="N28" t="str">
-        <v>1</v>
-      </c>
-      <c r="O28" t="str">
-        <v>46226</v>
-      </c>
-      <c r="P28" t="str">
-        <v/>
+        <v>26.7.2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O25"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K13"/>
+  <dimension ref="A1:K7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -6851,435 +6626,225 @@
         <v>Seller SKU ID</v>
       </c>
       <c r="J1" t="str">
-        <v>Юр Лицо</v>
+        <v>1</v>
       </c>
       <c r="K1" t="str">
-        <v>Дата</v>
+        <v>24.07.2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>SKU</v>
+        <v>АЛТЕЯ-PINKREM</v>
       </c>
       <c r="B2" t="str">
-        <v>Наименование</v>
+        <v>Крем для лица увлажняющий питательный с ниацинамидом Алтея 50 мл</v>
       </c>
       <c r="C2" t="str">
-        <v>Категория</v>
+        <v>1</v>
       </c>
       <c r="D2" t="str">
-        <v>Количество</v>
+        <v>0</v>
       </c>
       <c r="E2" t="str">
-        <v>Выручка (руб.)</v>
+        <v>437,95</v>
       </c>
       <c r="F2" t="str">
-        <v>Себестоимость (руб.)</v>
+        <v>147,85</v>
       </c>
       <c r="G2" t="str">
-        <v>Выручка с вычетом комиссии (руб.)</v>
+        <v>315,32</v>
       </c>
       <c r="H2" t="str">
-        <v>Комиссия маркетплейса(руб.)</v>
+        <v>122,63</v>
       </c>
       <c r="I2" t="str">
-        <v>Seller SKU ID</v>
+        <v>pink_pepper_50ml</v>
       </c>
       <c r="J2" t="str">
         <v>1</v>
       </c>
       <c r="K2" t="str">
-        <v>46226</v>
+        <v>24.07.2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>АЛТЕЯ-MASKARS</v>
+        <v>АЛТЕЯ-CUDRKRM</v>
       </c>
       <c r="B3" t="str">
-        <v>Маска для роста волос с перцем Алтея 500 мл</v>
+        <v>Крем для кудрявых и вьющихся волос Алтея 300 мл</v>
       </c>
       <c r="C3" t="str">
-        <v>Маски</v>
+        <v>3</v>
       </c>
       <c r="D3" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E3" t="str">
-        <v>384</v>
+        <v>1926</v>
       </c>
       <c r="F3" t="str">
-        <v>136.15</v>
+        <v>396</v>
       </c>
       <c r="G3" t="str">
-        <v>291.84</v>
+        <v>1386,72</v>
       </c>
       <c r="H3" t="str">
-        <v>92.16</v>
+        <v>539,28</v>
       </c>
       <c r="I3" t="str">
-        <v>maska-batter_dlya_rosta_500ml</v>
+        <v>curly_method_300ml</v>
       </c>
       <c r="J3" t="str">
         <v>1</v>
       </c>
       <c r="K3" t="str">
-        <v>46226</v>
+        <v>24.07.2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>АЛТЕЯ-CUDRKRM</v>
+        <v>АЛТЕЯ-ENZIMPD</v>
       </c>
       <c r="B4" t="str">
-        <v>Крем для кудрявых и вьющихся волос Алтея 300 мл</v>
+        <v>Энзимная пудра для умывания тела и лица от прыщей Алтея 80г</v>
       </c>
       <c r="C4" t="str">
-        <v>Кремы</v>
+        <v>1</v>
       </c>
       <c r="D4" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E4" t="str">
-        <v>642</v>
+        <v>431,3</v>
       </c>
       <c r="F4" t="str">
-        <v>132</v>
+        <v>114,6</v>
       </c>
       <c r="G4" t="str">
-        <v>462.24</v>
+        <v>310,54</v>
       </c>
       <c r="H4" t="str">
-        <v>179.76</v>
+        <v>120,76</v>
       </c>
       <c r="I4" t="str">
-        <v>curly_method_300ml</v>
+        <v>enzim_pudra_80gr</v>
       </c>
       <c r="J4" t="str">
         <v>1</v>
       </c>
       <c r="K4" t="str">
-        <v>46226</v>
+        <v>24.07.2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>АЛТЕЯ-KRRET15</v>
+        <v>АЛТЕЯ-KREMRST</v>
       </c>
       <c r="B5" t="str">
-        <v>Крем для лица с липосомальным ретинолом 1.5% Ретинайт</v>
+        <v>Крем масло от растяжек для беременных и подростков с эластином Алтея 200 мл</v>
       </c>
       <c r="C5" t="str">
-        <v>Кремы для лица</v>
+        <v>1</v>
       </c>
       <c r="D5" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>883.5</v>
+        <v>355</v>
       </c>
       <c r="F5" t="str">
-        <v>114.99</v>
+        <v>151,2</v>
       </c>
       <c r="G5" t="str">
-        <v>636.12</v>
+        <v>255,6</v>
       </c>
       <c r="H5" t="str">
-        <v>247.38</v>
+        <v>99,4</v>
       </c>
       <c r="I5" t="str">
-        <v>retinait_krem_1_5_50ml</v>
+        <v>krem_ot_rastyazhek</v>
       </c>
       <c r="J5" t="str">
         <v>1</v>
       </c>
       <c r="K5" t="str">
-        <v>46226</v>
+        <v>24.07.2026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>АЛТЕЯ-RETINT1</v>
+        <v>АЛТЕЯ-SYVTL30</v>
       </c>
       <c r="B6" t="str">
-        <v>Сыворотка с ретинолом 1% для лица от морщин антивозрастная Алтея 30 мл</v>
+        <v>Сыворотка для лица с ниацинамидом антивозрастная от акне пигментации Алтея 30 мл</v>
       </c>
       <c r="C6" t="str">
-        <v>Сыворотки</v>
+        <v>1</v>
       </c>
       <c r="D6" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E6" t="str">
-        <v>660</v>
+        <v>474,05</v>
       </c>
       <c r="F6" t="str">
-        <v>143.82</v>
+        <v>148,9</v>
       </c>
       <c r="G6" t="str">
-        <v>429</v>
+        <v>308,13</v>
       </c>
       <c r="H6" t="str">
-        <v>231</v>
+        <v>165,92</v>
       </c>
       <c r="I6" t="str">
-        <v>retinait_syvorotka_1_30ml</v>
+        <v>syvorotka_dlya_lica_30ml</v>
       </c>
       <c r="J6" t="str">
         <v>1</v>
       </c>
       <c r="K6" t="str">
-        <v>46226</v>
+        <v>24.07.2026</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>АЛТЕЯ-GELDLBR</v>
+        <v>АЛТЕЯ-SHPPERH</v>
       </c>
       <c r="B7" t="str">
-        <v>Гель для бритья мужской охлаждающий с ментолом Алтея 300 мл</v>
+        <v>Шампунь от перхоти лечебный с климбазолом Алтея 250 мл</v>
       </c>
       <c r="C7" t="str">
-        <v>Средства до и после бритья</v>
+        <v>1</v>
       </c>
       <c r="D7" t="str">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E7" t="str">
-        <v>522.5</v>
+        <v>428,45</v>
       </c>
       <c r="F7" t="str">
-        <v>125.68</v>
+        <v>106,2</v>
       </c>
       <c r="G7" t="str">
-        <v>376.2</v>
+        <v>308,48</v>
       </c>
       <c r="H7" t="str">
-        <v>146.3</v>
+        <v>119,97</v>
       </c>
       <c r="I7" t="str">
-        <v>gel_dlya_britya_300ml</v>
+        <v>shampun_protiv_perhoti_250ml</v>
       </c>
       <c r="J7" t="str">
         <v>1</v>
       </c>
       <c r="K7" t="str">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>АЛТЕЯ-PENKARS</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Пенка для нарощенных ресниц и для бровей для умывания и очищения ресниц Алтея 150 мл</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Пенка для умывания</v>
-      </c>
-      <c r="D8" t="str">
-        <v>1</v>
-      </c>
-      <c r="E8" t="str">
-        <v>558.6</v>
-      </c>
-      <c r="F8" t="str">
-        <v>90.65</v>
-      </c>
-      <c r="G8" t="str">
-        <v>363.09</v>
-      </c>
-      <c r="H8" t="str">
-        <v>195.51</v>
-      </c>
-      <c r="I8" t="str">
-        <v>nabor_penka_dlya_resnic</v>
-      </c>
-      <c r="J8" t="str">
-        <v>1</v>
-      </c>
-      <c r="K8" t="str">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>АЛТЕЯ-KREMRST</v>
-      </c>
-      <c r="B9" t="str">
-        <v>Крем масло от растяжек для беременных и подростков с эластином Алтея 200 мл</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Средство от растяжек</v>
-      </c>
-      <c r="D9" t="str">
-        <v>1</v>
-      </c>
-      <c r="E9" t="str">
-        <v>355</v>
-      </c>
-      <c r="F9" t="str">
-        <v>151.2</v>
-      </c>
-      <c r="G9" t="str">
-        <v>255.6</v>
-      </c>
-      <c r="H9" t="str">
-        <v>99.4</v>
-      </c>
-      <c r="I9" t="str">
-        <v>krem_ot_rastyazhek</v>
-      </c>
-      <c r="J9" t="str">
-        <v>1</v>
-      </c>
-      <c r="K9" t="str">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>SKU</v>
-      </c>
-      <c r="B10" t="str">
-        <v>Наименование</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Категория</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Количество</v>
-      </c>
-      <c r="E10" t="str">
-        <v>Выручка (руб.)</v>
-      </c>
-      <c r="F10" t="str">
-        <v>Себестоимость (руб.)</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Выручка с вычетом комиссии (руб.)</v>
-      </c>
-      <c r="H10" t="str">
-        <v>Комиссия маркетплейса(руб.)</v>
-      </c>
-      <c r="I10" t="str">
-        <v>Seller SKU ID</v>
-      </c>
-      <c r="J10" t="str">
-        <v>2</v>
-      </c>
-      <c r="K10" t="str">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>QEEP-ENZYMPD</v>
-      </c>
-      <c r="B11" t="str">
-        <v>Энзимная пудра для умывания лица и тела</v>
-      </c>
-      <c r="C11" t="str">
-        <v>1</v>
-      </c>
-      <c r="D11" t="str">
-        <v>0</v>
-      </c>
-      <c r="E11" t="str">
-        <v>511.1</v>
-      </c>
-      <c r="F11" t="str">
-        <v>119</v>
-      </c>
-      <c r="G11" t="str">
-        <v>367.99</v>
-      </c>
-      <c r="H11" t="str">
-        <v>143.11</v>
-      </c>
-      <c r="I11" t="str">
-        <v>qeep_enzyme_80g</v>
-      </c>
-      <c r="J11" t="str">
-        <v>2</v>
-      </c>
-      <c r="K11" t="str">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>QEEP-SYVORTV</v>
-      </c>
-      <c r="B12" t="str">
-        <v>Спрей для волос для роста и от выпадения волос qeep 100 мл</v>
-      </c>
-      <c r="C12" t="str">
-        <v>1</v>
-      </c>
-      <c r="D12" t="str">
-        <v>0</v>
-      </c>
-      <c r="E12" t="str">
-        <v>508.25</v>
-      </c>
-      <c r="F12" t="str">
-        <v>135.47</v>
-      </c>
-      <c r="G12" t="str">
-        <v>365.94</v>
-      </c>
-      <c r="H12" t="str">
-        <v>142.31</v>
-      </c>
-      <c r="I12" t="str">
-        <v>qeep_dlyarostavolos_100ml</v>
-      </c>
-      <c r="J12" t="str">
-        <v>2</v>
-      </c>
-      <c r="K12" t="str">
-        <v>46226</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>QEEP-KROVAVP</v>
-      </c>
-      <c r="B13" t="str">
-        <v>Кровавый кислотный пилинг для лица от прыщей с Альфа и бета-гидроксикислотами qeep 30 мл</v>
-      </c>
-      <c r="C13" t="str">
-        <v>1</v>
-      </c>
-      <c r="D13" t="str">
-        <v>0</v>
-      </c>
-      <c r="E13" t="str">
-        <v>550.05</v>
-      </c>
-      <c r="F13" t="str">
-        <v>105.2</v>
-      </c>
-      <c r="G13" t="str">
-        <v>357.53</v>
-      </c>
-      <c r="H13" t="str">
-        <v>192.52</v>
-      </c>
-      <c r="I13" t="str">
-        <v>qeep_bloodypeeling_30ml</v>
-      </c>
-      <c r="J13" t="str">
-        <v>2</v>
-      </c>
-      <c r="K13" t="str">
-        <v>46226</v>
+        <v>24.07.2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K13"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Refresh retail fallback through July 28
</commit_message>
<xml_diff>
--- a/data/external_sources/retail_network_sales.xlsx
+++ b/data/external_sources/retail_network_sales.xlsx
@@ -10630,7 +10630,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O25"/>
+  <dimension ref="A1:O28"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -10672,1151 +10672,1292 @@
       <c r="M1" t="str">
         <v>Возвраты шт</v>
       </c>
-      <c r="N1">
-        <v>2</v>
-      </c>
-      <c r="O1">
-        <v>46230</v>
+      <c r="N1" t="str">
+        <v>1</v>
+      </c>
+      <c r="O1" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
         <v>"Кровавый" пилинг для лица маркировки "Алтэя"</v>
       </c>
-      <c r="B2">
+      <c r="B2" t="str">
         <v>99000076205</v>
       </c>
       <c r="C2" t="str">
         <v>krovavii_piling_30ml</v>
       </c>
-      <c r="D2">
+      <c r="D2" t="str">
         <v>4670020498208</v>
       </c>
-      <c r="E2">
-        <v>9352</v>
-      </c>
-      <c r="F2">
-        <v>1336</v>
-      </c>
-      <c r="G2">
-        <v>8016</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2">
-        <v>14</v>
-      </c>
-      <c r="J2">
-        <v>2</v>
-      </c>
-      <c r="K2">
-        <v>12</v>
-      </c>
-      <c r="L2">
-        <v>0</v>
-      </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>1</v>
-      </c>
-      <c r="O2">
-        <v>46230</v>
+      <c r="E2" t="str">
+        <v>11985</v>
+      </c>
+      <c r="F2" t="str">
+        <v>668</v>
+      </c>
+      <c r="G2" t="str">
+        <v>11317</v>
+      </c>
+      <c r="H2" t="str">
+        <v>0</v>
+      </c>
+      <c r="I2" t="str">
+        <v>18</v>
+      </c>
+      <c r="J2" t="str">
+        <v>1</v>
+      </c>
+      <c r="K2" t="str">
+        <v>17</v>
+      </c>
+      <c r="L2" t="str">
+        <v>0</v>
+      </c>
+      <c r="M2" t="str">
+        <v>0</v>
+      </c>
+      <c r="N2" t="str">
+        <v>1</v>
+      </c>
+      <c r="O2" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Гель для проблемной кожи лица и тела, с маркировками Алтея</v>
-      </c>
-      <c r="B3">
-        <v>99000114730</v>
+        <v>Крем для волос Упругий завиток, 300 мл</v>
+      </c>
+      <c r="B3" t="str">
+        <v>99000114726</v>
       </c>
       <c r="C3" t="str">
-        <v>gel_antiakne_20ml_v2</v>
-      </c>
-      <c r="D3">
-        <v>4660417420110</v>
-      </c>
-      <c r="E3">
-        <v>7928</v>
-      </c>
-      <c r="F3">
-        <v>856</v>
-      </c>
-      <c r="G3">
-        <v>7072</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3">
-        <v>19</v>
-      </c>
-      <c r="J3">
-        <v>2</v>
-      </c>
-      <c r="K3">
-        <v>17</v>
-      </c>
-      <c r="L3">
-        <v>0</v>
-      </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>1</v>
-      </c>
-      <c r="O3">
-        <v>46230</v>
+        <v>curly_method_300ml</v>
+      </c>
+      <c r="D3" t="str">
+        <v>4603320465441</v>
+      </c>
+      <c r="E3" t="str">
+        <v>8424</v>
+      </c>
+      <c r="F3" t="str">
+        <v>903</v>
+      </c>
+      <c r="G3" t="str">
+        <v>7521</v>
+      </c>
+      <c r="H3" t="str">
+        <v>0</v>
+      </c>
+      <c r="I3" t="str">
+        <v>10</v>
+      </c>
+      <c r="J3" t="str">
+        <v>1</v>
+      </c>
+      <c r="K3" t="str">
+        <v>9</v>
+      </c>
+      <c r="L3" t="str">
+        <v>0</v>
+      </c>
+      <c r="M3" t="str">
+        <v>0</v>
+      </c>
+      <c r="N3" t="str">
+        <v>1</v>
+      </c>
+      <c r="O3" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Крем для волос Упругий завиток, 300 мл</v>
-      </c>
-      <c r="B4">
-        <v>99000114726</v>
+        <v>Гель для проблемной кожи лица и тела, с маркировками Алтея</v>
+      </c>
+      <c r="B4" t="str">
+        <v>99000114730</v>
       </c>
       <c r="C4" t="str">
-        <v>curly_method_300ml</v>
-      </c>
-      <c r="D4">
-        <v>4603320465441</v>
-      </c>
-      <c r="E4">
-        <v>6718</v>
-      </c>
-      <c r="F4">
-        <v>2203</v>
-      </c>
-      <c r="G4">
-        <v>4515</v>
-      </c>
-      <c r="H4">
-        <v>0</v>
-      </c>
-      <c r="I4">
-        <v>8</v>
-      </c>
-      <c r="J4">
-        <v>3</v>
-      </c>
-      <c r="K4">
-        <v>5</v>
-      </c>
-      <c r="L4">
-        <v>0</v>
-      </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>1</v>
-      </c>
-      <c r="O4">
-        <v>46230</v>
+        <v>gel_antiakne_20ml_v2</v>
+      </c>
+      <c r="D4" t="str">
+        <v>4660417420110</v>
+      </c>
+      <c r="E4" t="str">
+        <v>7893</v>
+      </c>
+      <c r="F4" t="str">
+        <v>0</v>
+      </c>
+      <c r="G4" t="str">
+        <v>7446</v>
+      </c>
+      <c r="H4" t="str">
+        <v>447</v>
+      </c>
+      <c r="I4" t="str">
+        <v>18</v>
+      </c>
+      <c r="J4" t="str">
+        <v>0</v>
+      </c>
+      <c r="K4" t="str">
+        <v>17</v>
+      </c>
+      <c r="L4" t="str">
+        <v>1</v>
+      </c>
+      <c r="M4" t="str">
+        <v>0</v>
+      </c>
+      <c r="N4" t="str">
+        <v>1</v>
+      </c>
+      <c r="O4" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>Продукция косметическая для ухода за кожей, в том числе в наборах: Маска для проблемной кожи лица м</v>
       </c>
-      <c r="B5">
+      <c r="B5" t="str">
         <v>99000114727</v>
       </c>
       <c r="C5" t="str">
         <v>maska_dlya_lica_100m</v>
       </c>
-      <c r="D5">
+      <c r="D5" t="str">
         <v>4670020498741</v>
       </c>
-      <c r="E5">
-        <v>6213</v>
-      </c>
-      <c r="F5">
-        <v>933</v>
-      </c>
-      <c r="G5">
-        <v>4341</v>
-      </c>
-      <c r="H5">
+      <c r="E5" t="str">
+        <v>7428</v>
+      </c>
+      <c r="F5" t="str">
+        <v>0</v>
+      </c>
+      <c r="G5" t="str">
+        <v>6489</v>
+      </c>
+      <c r="H5" t="str">
         <v>939</v>
       </c>
-      <c r="I5">
+      <c r="I5" t="str">
+        <v>8</v>
+      </c>
+      <c r="J5" t="str">
+        <v>0</v>
+      </c>
+      <c r="K5" t="str">
         <v>7</v>
       </c>
-      <c r="J5">
-        <v>1</v>
-      </c>
-      <c r="K5">
-        <v>5</v>
-      </c>
-      <c r="L5">
-        <v>1</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>1</v>
-      </c>
-      <c r="O5">
-        <v>46230</v>
+      <c r="L5" t="str">
+        <v>1</v>
+      </c>
+      <c r="M5" t="str">
+        <v>0</v>
+      </c>
+      <c r="N5" t="str">
+        <v>1</v>
+      </c>
+      <c r="O5" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Крем для лица с ретинолом 0.5, сыворотка от морщин и пигментных пятен, Алтея, Ретидерм, 50 мл</v>
-      </c>
-      <c r="B6">
-        <v>99000076216</v>
+        <v>Пенка для укладки волос</v>
+      </c>
+      <c r="B6" t="str">
+        <v>99000125266</v>
       </c>
       <c r="C6" t="str">
-        <v>retiderm_50ml</v>
-      </c>
-      <c r="D6">
-        <v>4610172186219</v>
-      </c>
-      <c r="E6">
-        <v>6195</v>
-      </c>
-      <c r="F6">
-        <v>1502</v>
-      </c>
-      <c r="G6">
-        <v>4693</v>
-      </c>
-      <c r="H6">
-        <v>0</v>
-      </c>
-      <c r="I6">
-        <v>26</v>
-      </c>
-      <c r="J6">
-        <v>6</v>
-      </c>
-      <c r="K6">
-        <v>20</v>
-      </c>
-      <c r="L6">
-        <v>0</v>
-      </c>
-      <c r="M6">
-        <v>0</v>
-      </c>
-      <c r="N6">
-        <v>1</v>
-      </c>
-      <c r="O6">
-        <v>46230</v>
+        <v>penka_kudryavii_meto</v>
+      </c>
+      <c r="D6" t="str">
+        <v>4670020498611</v>
+      </c>
+      <c r="E6" t="str">
+        <v>6242</v>
+      </c>
+      <c r="F6" t="str">
+        <v>0</v>
+      </c>
+      <c r="G6" t="str">
+        <v>6242</v>
+      </c>
+      <c r="H6" t="str">
+        <v>0</v>
+      </c>
+      <c r="I6" t="str">
+        <v>9</v>
+      </c>
+      <c r="J6" t="str">
+        <v>0</v>
+      </c>
+      <c r="K6" t="str">
+        <v>9</v>
+      </c>
+      <c r="L6" t="str">
+        <v>0</v>
+      </c>
+      <c r="M6" t="str">
+        <v>0</v>
+      </c>
+      <c r="N6" t="str">
+        <v>1</v>
+      </c>
+      <c r="O6" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Пенка для укладки волос</v>
-      </c>
-      <c r="B7">
-        <v>99000125266</v>
+        <v>Крем специального назначения «Псоридонт» 50 мл</v>
+      </c>
+      <c r="B7" t="str">
+        <v>99000125141</v>
       </c>
       <c r="C7" t="str">
-        <v>penka_kudryavii_meto</v>
-      </c>
-      <c r="D7">
-        <v>4670020498611</v>
-      </c>
-      <c r="E7">
-        <v>5581</v>
-      </c>
-      <c r="F7">
-        <v>1081</v>
-      </c>
-      <c r="G7">
-        <v>4500</v>
-      </c>
-      <c r="H7">
-        <v>0</v>
-      </c>
-      <c r="I7">
-        <v>8</v>
-      </c>
-      <c r="J7">
-        <v>2</v>
-      </c>
-      <c r="K7">
-        <v>6</v>
-      </c>
-      <c r="L7">
-        <v>0</v>
-      </c>
-      <c r="M7">
-        <v>0</v>
-      </c>
-      <c r="N7">
-        <v>1</v>
-      </c>
-      <c r="O7">
-        <v>46230</v>
+        <v>psoral_50ml</v>
+      </c>
+      <c r="D7" t="str">
+        <v>4660417421087</v>
+      </c>
+      <c r="E7" t="str">
+        <v>5112</v>
+      </c>
+      <c r="F7" t="str">
+        <v>0</v>
+      </c>
+      <c r="G7" t="str">
+        <v>5112</v>
+      </c>
+      <c r="H7" t="str">
+        <v>0</v>
+      </c>
+      <c r="I7" t="str">
+        <v>7</v>
+      </c>
+      <c r="J7" t="str">
+        <v>0</v>
+      </c>
+      <c r="K7" t="str">
+        <v>7</v>
+      </c>
+      <c r="L7" t="str">
+        <v>0</v>
+      </c>
+      <c r="M7" t="str">
+        <v>0</v>
+      </c>
+      <c r="N7" t="str">
+        <v>1</v>
+      </c>
+      <c r="O7" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Крем-шелк для сухой кожи ног</v>
-      </c>
-      <c r="B8">
-        <v>99000076225</v>
+        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея</v>
+      </c>
+      <c r="B8" t="str">
+        <v>99000124421</v>
       </c>
       <c r="C8" t="str">
-        <v>kremshelk_100ml</v>
-      </c>
-      <c r="D8">
-        <v>4670020498437</v>
-      </c>
-      <c r="E8">
-        <v>3776</v>
-      </c>
-      <c r="F8">
-        <v>1806</v>
-      </c>
-      <c r="G8">
-        <v>1970</v>
-      </c>
-      <c r="H8">
-        <v>0</v>
-      </c>
-      <c r="I8">
-        <v>8</v>
-      </c>
-      <c r="J8">
+        <v>retinait_krem_1_50ml</v>
+      </c>
+      <c r="D8" t="str">
+        <v>4660417421605</v>
+      </c>
+      <c r="E8" t="str">
+        <v>5046</v>
+      </c>
+      <c r="F8" t="str">
+        <v>1025</v>
+      </c>
+      <c r="G8" t="str">
+        <v>4021</v>
+      </c>
+      <c r="H8" t="str">
+        <v>0</v>
+      </c>
+      <c r="I8" t="str">
+        <v>5</v>
+      </c>
+      <c r="J8" t="str">
+        <v>1</v>
+      </c>
+      <c r="K8" t="str">
         <v>4</v>
       </c>
-      <c r="K8">
-        <v>4</v>
-      </c>
-      <c r="L8">
-        <v>0</v>
-      </c>
-      <c r="M8">
-        <v>0</v>
-      </c>
-      <c r="N8">
-        <v>1</v>
-      </c>
-      <c r="O8">
-        <v>46230</v>
+      <c r="L8" t="str">
+        <v>0</v>
+      </c>
+      <c r="M8" t="str">
+        <v>0</v>
+      </c>
+      <c r="N8" t="str">
+        <v>1</v>
+      </c>
+      <c r="O8" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея</v>
-      </c>
-      <c r="B9">
-        <v>99000124421</v>
+        <v>Спрей для роста волос торговой марки Алтея</v>
+      </c>
+      <c r="B9" t="str">
+        <v>99000114724</v>
       </c>
       <c r="C9" t="str">
-        <v>retinait_krem_1_50ml</v>
-      </c>
-      <c r="D9">
-        <v>4660417421605</v>
-      </c>
-      <c r="E9">
-        <v>3075</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9">
-        <v>3075</v>
-      </c>
-      <c r="H9">
-        <v>0</v>
-      </c>
-      <c r="I9">
-        <v>3</v>
-      </c>
-      <c r="J9">
-        <v>0</v>
-      </c>
-      <c r="K9">
-        <v>3</v>
-      </c>
-      <c r="L9">
-        <v>0</v>
-      </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
-        <v>1</v>
-      </c>
-      <c r="O9">
-        <v>46230</v>
+        <v>sprei_buster_100ml</v>
+      </c>
+      <c r="D9" t="str">
+        <v>4603320465359</v>
+      </c>
+      <c r="E9" t="str">
+        <v>4211</v>
+      </c>
+      <c r="F9" t="str">
+        <v>602</v>
+      </c>
+      <c r="G9" t="str">
+        <v>3609</v>
+      </c>
+      <c r="H9" t="str">
+        <v>0</v>
+      </c>
+      <c r="I9" t="str">
+        <v>7</v>
+      </c>
+      <c r="J9" t="str">
+        <v>1</v>
+      </c>
+      <c r="K9" t="str">
+        <v>6</v>
+      </c>
+      <c r="L9" t="str">
+        <v>0</v>
+      </c>
+      <c r="M9" t="str">
+        <v>0</v>
+      </c>
+      <c r="N9" t="str">
+        <v>1</v>
+      </c>
+      <c r="O9" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>Крем от растяжек, Алтея, 200 мл</v>
-      </c>
-      <c r="B10">
-        <v>99000114731</v>
+        <v>Продукция косметическая для ухода за кожей для взрослых: гелевая маска со спикулами торговой марки А</v>
+      </c>
+      <c r="B10" t="str">
+        <v>99000177799</v>
       </c>
       <c r="C10" t="str">
-        <v>krem_ot_rastyazhek</v>
-      </c>
-      <c r="D10">
-        <v>4670020497898</v>
-      </c>
-      <c r="E10">
-        <v>2960</v>
-      </c>
-      <c r="F10">
-        <v>1654</v>
-      </c>
-      <c r="G10">
-        <v>1306</v>
-      </c>
-      <c r="H10">
-        <v>0</v>
-      </c>
-      <c r="I10">
-        <v>4</v>
-      </c>
-      <c r="J10">
-        <v>2</v>
-      </c>
-      <c r="K10">
-        <v>2</v>
-      </c>
-      <c r="L10">
-        <v>0</v>
-      </c>
-      <c r="M10">
-        <v>0</v>
-      </c>
-      <c r="N10">
-        <v>1</v>
-      </c>
-      <c r="O10">
-        <v>46230</v>
+        <v>spicul_gel_mask_75ml</v>
+      </c>
+      <c r="D10" t="str">
+        <v>4660417421858</v>
+      </c>
+      <c r="E10" t="str">
+        <v>4208</v>
+      </c>
+      <c r="F10" t="str">
+        <v>0</v>
+      </c>
+      <c r="G10" t="str">
+        <v>4208</v>
+      </c>
+      <c r="H10" t="str">
+        <v>0</v>
+      </c>
+      <c r="I10" t="str">
+        <v>5</v>
+      </c>
+      <c r="J10" t="str">
+        <v>0</v>
+      </c>
+      <c r="K10" t="str">
+        <v>5</v>
+      </c>
+      <c r="L10" t="str">
+        <v>0</v>
+      </c>
+      <c r="M10" t="str">
+        <v>0</v>
+      </c>
+      <c r="N10" t="str">
+        <v>1</v>
+      </c>
+      <c r="O10" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>Спрей-сыворотка для волос маркировки Алтея</v>
-      </c>
-      <c r="B11">
-        <v>99000076226</v>
+        <v>Крем для лица с ретинолом 0.5, сыворотка от морщин и пигментных пятен, Алтея, Ретидерм, 50 мл</v>
+      </c>
+      <c r="B11" t="str">
+        <v>99000076216</v>
       </c>
       <c r="C11" t="str">
-        <v>termo_sprei_200ml</v>
-      </c>
-      <c r="D11">
-        <v>4670020497980</v>
-      </c>
-      <c r="E11">
-        <v>2614</v>
-      </c>
-      <c r="F11">
-        <v>472</v>
-      </c>
-      <c r="G11">
-        <v>1683</v>
-      </c>
-      <c r="H11">
-        <v>459</v>
-      </c>
-      <c r="I11">
-        <v>6</v>
-      </c>
-      <c r="J11">
-        <v>1</v>
-      </c>
-      <c r="K11">
-        <v>4</v>
-      </c>
-      <c r="L11">
-        <v>1</v>
-      </c>
-      <c r="M11">
-        <v>0</v>
-      </c>
-      <c r="N11">
-        <v>1</v>
-      </c>
-      <c r="O11">
-        <v>46230</v>
+        <v>retiderm_50ml</v>
+      </c>
+      <c r="D11" t="str">
+        <v>4610172186219</v>
+      </c>
+      <c r="E11" t="str">
+        <v>3821</v>
+      </c>
+      <c r="F11" t="str">
+        <v>0</v>
+      </c>
+      <c r="G11" t="str">
+        <v>3821</v>
+      </c>
+      <c r="H11" t="str">
+        <v>0</v>
+      </c>
+      <c r="I11" t="str">
+        <v>17</v>
+      </c>
+      <c r="J11" t="str">
+        <v>0</v>
+      </c>
+      <c r="K11" t="str">
+        <v>17</v>
+      </c>
+      <c r="L11" t="str">
+        <v>0</v>
+      </c>
+      <c r="M11" t="str">
+        <v>0</v>
+      </c>
+      <c r="N11" t="str">
+        <v>1</v>
+      </c>
+      <c r="O11" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>Средство косметическое: Воск для волос торговой марки: «Алтея» 15гр</v>
-      </c>
-      <c r="B12">
-        <v>99000131672</v>
+        <v>Крем от растяжек, Алтея, 200 мл</v>
+      </c>
+      <c r="B12" t="str">
+        <v>99000114731</v>
       </c>
       <c r="C12" t="str">
-        <v>vosk_stik_15ml</v>
-      </c>
-      <c r="D12">
-        <v>4670207150196</v>
-      </c>
-      <c r="E12">
-        <v>2573</v>
-      </c>
-      <c r="F12">
-        <v>0</v>
-      </c>
-      <c r="G12">
-        <v>2573</v>
-      </c>
-      <c r="H12">
-        <v>0</v>
-      </c>
-      <c r="I12">
-        <v>6</v>
-      </c>
-      <c r="J12">
-        <v>0</v>
-      </c>
-      <c r="K12">
-        <v>6</v>
-      </c>
-      <c r="L12">
-        <v>0</v>
-      </c>
-      <c r="M12">
-        <v>0</v>
-      </c>
-      <c r="N12">
-        <v>1</v>
-      </c>
-      <c r="O12">
-        <v>46230</v>
+        <v>krem_ot_rastyazhek</v>
+      </c>
+      <c r="D12" t="str">
+        <v>4670020497898</v>
+      </c>
+      <c r="E12" t="str">
+        <v>3102</v>
+      </c>
+      <c r="F12" t="str">
+        <v>0</v>
+      </c>
+      <c r="G12" t="str">
+        <v>3102</v>
+      </c>
+      <c r="H12" t="str">
+        <v>0</v>
+      </c>
+      <c r="I12" t="str">
+        <v>4</v>
+      </c>
+      <c r="J12" t="str">
+        <v>0</v>
+      </c>
+      <c r="K12" t="str">
+        <v>4</v>
+      </c>
+      <c r="L12" t="str">
+        <v>0</v>
+      </c>
+      <c r="M12" t="str">
+        <v>0</v>
+      </c>
+      <c r="N12" t="str">
+        <v>1</v>
+      </c>
+      <c r="O12" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>Продукция косметическая для ухода за кожей для взрослых: гелевая маска со спикулами торговой марки А</v>
-      </c>
-      <c r="B13">
-        <v>99000177799</v>
+        <v>Крем c ретинолом для век антивозрастной для кожи и кожи вокруг глаз, 30мл</v>
+      </c>
+      <c r="B13" t="str">
+        <v>99000154005</v>
       </c>
       <c r="C13" t="str">
-        <v>spicul_gel_mask_75ml</v>
-      </c>
-      <c r="D13">
-        <v>4660417421858</v>
-      </c>
-      <c r="E13">
-        <v>2523</v>
-      </c>
-      <c r="F13">
-        <v>829</v>
-      </c>
-      <c r="G13">
-        <v>1694</v>
-      </c>
-      <c r="H13">
-        <v>0</v>
-      </c>
-      <c r="I13">
+        <v>retinol_boost_krem_d</v>
+      </c>
+      <c r="D13" t="str">
+        <v>4660417421636</v>
+      </c>
+      <c r="E13" t="str">
+        <v>2625</v>
+      </c>
+      <c r="F13" t="str">
+        <v>893</v>
+      </c>
+      <c r="G13" t="str">
+        <v>1732</v>
+      </c>
+      <c r="H13" t="str">
+        <v>0</v>
+      </c>
+      <c r="I13" t="str">
         <v>3</v>
       </c>
-      <c r="J13">
-        <v>1</v>
-      </c>
-      <c r="K13">
+      <c r="J13" t="str">
+        <v>1</v>
+      </c>
+      <c r="K13" t="str">
         <v>2</v>
       </c>
-      <c r="L13">
-        <v>0</v>
-      </c>
-      <c r="M13">
-        <v>0</v>
-      </c>
-      <c r="N13">
-        <v>1</v>
-      </c>
-      <c r="O13">
-        <v>46230</v>
+      <c r="L13" t="str">
+        <v>0</v>
+      </c>
+      <c r="M13" t="str">
+        <v>0</v>
+      </c>
+      <c r="N13" t="str">
+        <v>1</v>
+      </c>
+      <c r="O13" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>Спрей для роста волос торговой марки Алтея</v>
-      </c>
-      <c r="B14">
-        <v>99000114724</v>
+        <v>Спрей-сыворотка для волос маркировки Алтея</v>
+      </c>
+      <c r="B14" t="str">
+        <v>99000076226</v>
       </c>
       <c r="C14" t="str">
-        <v>sprei_buster_100ml</v>
-      </c>
-      <c r="D14">
-        <v>4603320465359</v>
-      </c>
-      <c r="E14">
-        <v>2391</v>
-      </c>
-      <c r="F14">
-        <v>602</v>
-      </c>
-      <c r="G14">
-        <v>1789</v>
-      </c>
-      <c r="H14">
-        <v>0</v>
-      </c>
-      <c r="I14">
-        <v>4</v>
-      </c>
-      <c r="J14">
-        <v>1</v>
-      </c>
-      <c r="K14">
-        <v>3</v>
-      </c>
-      <c r="L14">
-        <v>0</v>
-      </c>
-      <c r="M14">
-        <v>0</v>
-      </c>
-      <c r="N14">
-        <v>1</v>
-      </c>
-      <c r="O14">
-        <v>46230</v>
+        <v>termo_sprei_200ml</v>
+      </c>
+      <c r="D14" t="str">
+        <v>4670020497980</v>
+      </c>
+      <c r="E14" t="str">
+        <v>2344</v>
+      </c>
+      <c r="F14" t="str">
+        <v>0</v>
+      </c>
+      <c r="G14" t="str">
+        <v>2344</v>
+      </c>
+      <c r="H14" t="str">
+        <v>0</v>
+      </c>
+      <c r="I14" t="str">
+        <v>5</v>
+      </c>
+      <c r="J14" t="str">
+        <v>0</v>
+      </c>
+      <c r="K14" t="str">
+        <v>5</v>
+      </c>
+      <c r="L14" t="str">
+        <v>0</v>
+      </c>
+      <c r="M14" t="str">
+        <v>0</v>
+      </c>
+      <c r="N14" t="str">
+        <v>1</v>
+      </c>
+      <c r="O14" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>Ламеллярный крем для рук с мочевиной, увлажняющий и питательный с маслом кокоса, Алтея, 75 мл</v>
-      </c>
-      <c r="B15">
-        <v>99000114729</v>
+        <v>Шампунь для кудрявых волос торговой марки Алтея, 500 мл</v>
+      </c>
+      <c r="B15" t="str">
+        <v>99000179424</v>
       </c>
       <c r="C15" t="str">
-        <v>krem_dlya_ruk_75ml</v>
-      </c>
-      <c r="D15">
-        <v>4660417421452</v>
-      </c>
-      <c r="E15">
-        <v>1545</v>
-      </c>
-      <c r="F15">
-        <v>1164</v>
-      </c>
-      <c r="G15">
-        <v>381</v>
-      </c>
-      <c r="H15">
-        <v>0</v>
-      </c>
-      <c r="I15">
-        <v>4</v>
-      </c>
-      <c r="J15">
-        <v>3</v>
-      </c>
-      <c r="K15">
-        <v>1</v>
-      </c>
-      <c r="L15">
-        <v>0</v>
-      </c>
-      <c r="M15">
-        <v>0</v>
-      </c>
-      <c r="N15">
-        <v>1</v>
-      </c>
-      <c r="O15">
-        <v>46230</v>
+        <v>shampun_kudryavii_me</v>
+      </c>
+      <c r="D15" t="str">
+        <v>4640523970310</v>
+      </c>
+      <c r="E15" t="str">
+        <v>1718</v>
+      </c>
+      <c r="F15" t="str">
+        <v>859</v>
+      </c>
+      <c r="G15" t="str">
+        <v>859</v>
+      </c>
+      <c r="H15" t="str">
+        <v>0</v>
+      </c>
+      <c r="I15" t="str">
+        <v>2</v>
+      </c>
+      <c r="J15" t="str">
+        <v>1</v>
+      </c>
+      <c r="K15" t="str">
+        <v>1</v>
+      </c>
+      <c r="L15" t="str">
+        <v>0</v>
+      </c>
+      <c r="M15" t="str">
+        <v>0</v>
+      </c>
+      <c r="N15" t="str">
+        <v>1</v>
+      </c>
+      <c r="O15" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>Крем c ретинолом для век антивозрастной для кожи и кожи вокруг глаз, 30мл</v>
-      </c>
-      <c r="B16">
-        <v>99000154005</v>
+        <v>Крем для лица spf 50 с защитой UVA/UVB, торговой марки Алтея</v>
+      </c>
+      <c r="B16" t="str">
+        <v>99000163832</v>
       </c>
       <c r="C16" t="str">
-        <v>retinol_boost_krem_d</v>
-      </c>
-      <c r="D16">
-        <v>4660417421636</v>
-      </c>
-      <c r="E16">
-        <v>893</v>
-      </c>
-      <c r="F16">
-        <v>0</v>
-      </c>
-      <c r="G16">
-        <v>893</v>
-      </c>
-      <c r="H16">
-        <v>0</v>
-      </c>
-      <c r="I16">
-        <v>1</v>
-      </c>
-      <c r="J16">
-        <v>0</v>
-      </c>
-      <c r="K16">
-        <v>1</v>
-      </c>
-      <c r="L16">
-        <v>0</v>
-      </c>
-      <c r="M16">
-        <v>0</v>
-      </c>
-      <c r="N16">
-        <v>1</v>
-      </c>
-      <c r="O16">
-        <v>46230</v>
+        <v>krem_spf50_50ml</v>
+      </c>
+      <c r="D16" t="str">
+        <v>4660417421766</v>
+      </c>
+      <c r="E16" t="str">
+        <v>1600</v>
+      </c>
+      <c r="F16" t="str">
+        <v>0</v>
+      </c>
+      <c r="G16" t="str">
+        <v>1600</v>
+      </c>
+      <c r="H16" t="str">
+        <v>0</v>
+      </c>
+      <c r="I16" t="str">
+        <v>2</v>
+      </c>
+      <c r="J16" t="str">
+        <v>0</v>
+      </c>
+      <c r="K16" t="str">
+        <v>2</v>
+      </c>
+      <c r="L16" t="str">
+        <v>0</v>
+      </c>
+      <c r="M16" t="str">
+        <v>0</v>
+      </c>
+      <c r="N16" t="str">
+        <v>1</v>
+      </c>
+      <c r="O16" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея</v>
-      </c>
-      <c r="B17">
-        <v>99000124418</v>
+        <v>Средство косметическое: Воск для волос торговой марки: «Алтея» 15гр</v>
+      </c>
+      <c r="B17" t="str">
+        <v>99000131672</v>
       </c>
       <c r="C17" t="str">
-        <v>retinait_krem_025_50</v>
-      </c>
-      <c r="D17">
-        <v>4660417421599</v>
-      </c>
-      <c r="E17">
-        <v>844</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-      <c r="G17">
-        <v>844</v>
-      </c>
-      <c r="H17">
-        <v>0</v>
-      </c>
-      <c r="I17">
-        <v>1</v>
-      </c>
-      <c r="J17">
-        <v>0</v>
-      </c>
-      <c r="K17">
-        <v>1</v>
-      </c>
-      <c r="L17">
-        <v>0</v>
-      </c>
-      <c r="M17">
-        <v>0</v>
-      </c>
-      <c r="N17">
-        <v>1</v>
-      </c>
-      <c r="O17">
-        <v>46230</v>
+        <v>vosk_stik_15ml</v>
+      </c>
+      <c r="D17" t="str">
+        <v>4670207150196</v>
+      </c>
+      <c r="E17" t="str">
+        <v>1432</v>
+      </c>
+      <c r="F17" t="str">
+        <v>0</v>
+      </c>
+      <c r="G17" t="str">
+        <v>1432</v>
+      </c>
+      <c r="H17" t="str">
+        <v>0</v>
+      </c>
+      <c r="I17" t="str">
+        <v>3</v>
+      </c>
+      <c r="J17" t="str">
+        <v>0</v>
+      </c>
+      <c r="K17" t="str">
+        <v>3</v>
+      </c>
+      <c r="L17" t="str">
+        <v>0</v>
+      </c>
+      <c r="M17" t="str">
+        <v>0</v>
+      </c>
+      <c r="N17" t="str">
+        <v>1</v>
+      </c>
+      <c r="O17" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>Крем для лица spf 50 с защитой UVA/UVB, торговой марки Алтея</v>
-      </c>
-      <c r="B18">
-        <v>99000163832</v>
+        <v>Средство косметическое для ухода за волосами: маска для волос восстанавливающая с авокадо и маслом о</v>
+      </c>
+      <c r="B18" t="str">
+        <v>99000076210</v>
       </c>
       <c r="C18" t="str">
-        <v>krem_spf50_50ml</v>
-      </c>
-      <c r="D18">
-        <v>4660417421766</v>
-      </c>
-      <c r="E18">
-        <v>800</v>
-      </c>
-      <c r="F18">
-        <v>800</v>
-      </c>
-      <c r="G18">
-        <v>0</v>
-      </c>
-      <c r="H18">
-        <v>0</v>
-      </c>
-      <c r="I18">
-        <v>1</v>
-      </c>
-      <c r="J18">
-        <v>1</v>
-      </c>
-      <c r="K18">
-        <v>0</v>
-      </c>
-      <c r="L18">
-        <v>0</v>
-      </c>
-      <c r="M18">
-        <v>0</v>
-      </c>
-      <c r="N18">
-        <v>1</v>
-      </c>
-      <c r="O18">
-        <v>46230</v>
+        <v>maska-batter_250ml</v>
+      </c>
+      <c r="D18" t="str">
+        <v>4670020497546</v>
+      </c>
+      <c r="E18" t="str">
+        <v>1376</v>
+      </c>
+      <c r="F18" t="str">
+        <v>0</v>
+      </c>
+      <c r="G18" t="str">
+        <v>1376</v>
+      </c>
+      <c r="H18" t="str">
+        <v>0</v>
+      </c>
+      <c r="I18" t="str">
+        <v>2</v>
+      </c>
+      <c r="J18" t="str">
+        <v>0</v>
+      </c>
+      <c r="K18" t="str">
+        <v>2</v>
+      </c>
+      <c r="L18" t="str">
+        <v>0</v>
+      </c>
+      <c r="M18" t="str">
+        <v>0</v>
+      </c>
+      <c r="N18" t="str">
+        <v>1</v>
+      </c>
+      <c r="O18" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>Крем специального назначения «Псоридонт» 50 мл</v>
-      </c>
-      <c r="B19">
-        <v>99000125141</v>
+        <v>Крем-шелк для сухой кожи ног</v>
+      </c>
+      <c r="B19" t="str">
+        <v>99000076225</v>
       </c>
       <c r="C19" t="str">
-        <v>psoral_50ml</v>
-      </c>
-      <c r="D19">
-        <v>4660417421087</v>
-      </c>
-      <c r="E19">
-        <v>760</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-      <c r="G19">
-        <v>760</v>
-      </c>
-      <c r="H19">
-        <v>0</v>
-      </c>
-      <c r="I19">
-        <v>1</v>
-      </c>
-      <c r="J19">
-        <v>0</v>
-      </c>
-      <c r="K19">
-        <v>1</v>
-      </c>
-      <c r="L19">
-        <v>0</v>
-      </c>
-      <c r="M19">
-        <v>0</v>
-      </c>
-      <c r="N19">
-        <v>1</v>
-      </c>
-      <c r="O19">
-        <v>46230</v>
+        <v>kremshelk_100ml</v>
+      </c>
+      <c r="D19" t="str">
+        <v>4670020498437</v>
+      </c>
+      <c r="E19" t="str">
+        <v>1335</v>
+      </c>
+      <c r="F19" t="str">
+        <v>0</v>
+      </c>
+      <c r="G19" t="str">
+        <v>1335</v>
+      </c>
+      <c r="H19" t="str">
+        <v>0</v>
+      </c>
+      <c r="I19" t="str">
+        <v>3</v>
+      </c>
+      <c r="J19" t="str">
+        <v>0</v>
+      </c>
+      <c r="K19" t="str">
+        <v>3</v>
+      </c>
+      <c r="L19" t="str">
+        <v>0</v>
+      </c>
+      <c r="M19" t="str">
+        <v>0</v>
+      </c>
+      <c r="N19" t="str">
+        <v>1</v>
+      </c>
+      <c r="O19" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>Ретинайт 0,5 экспресс-омоложение Anti-Age Липосомальный комплекс ретинола 0,5 + Ниацинамид 50 мл</v>
-      </c>
-      <c r="B20">
-        <v>99000131675</v>
+        <v>Маска д/лица Лифтинг PDRN и пептиды 75мл</v>
+      </c>
+      <c r="B20" t="str">
+        <v>99000188068</v>
       </c>
       <c r="C20" t="str">
-        <v>retinait_krem_05_50m</v>
-      </c>
-      <c r="D20">
-        <v>4660417421759</v>
-      </c>
-      <c r="E20">
-        <v>744</v>
-      </c>
-      <c r="F20">
-        <v>0</v>
-      </c>
-      <c r="G20">
-        <v>744</v>
-      </c>
-      <c r="H20">
-        <v>0</v>
-      </c>
-      <c r="I20">
-        <v>1</v>
-      </c>
-      <c r="J20">
-        <v>0</v>
-      </c>
-      <c r="K20">
-        <v>1</v>
-      </c>
-      <c r="L20">
-        <v>0</v>
-      </c>
-      <c r="M20">
-        <v>0</v>
-      </c>
-      <c r="N20">
-        <v>1</v>
-      </c>
-      <c r="O20">
-        <v>46230</v>
+        <v>lifting_maska_pdrn_7</v>
+      </c>
+      <c r="D20" t="str">
+        <v>4660417421964</v>
+      </c>
+      <c r="E20" t="str">
+        <v>1165</v>
+      </c>
+      <c r="F20" t="str">
+        <v>0</v>
+      </c>
+      <c r="G20" t="str">
+        <v>1165</v>
+      </c>
+      <c r="H20" t="str">
+        <v>0</v>
+      </c>
+      <c r="I20" t="str">
+        <v>1</v>
+      </c>
+      <c r="J20" t="str">
+        <v>0</v>
+      </c>
+      <c r="K20" t="str">
+        <v>1</v>
+      </c>
+      <c r="L20" t="str">
+        <v>0</v>
+      </c>
+      <c r="M20" t="str">
+        <v>0</v>
+      </c>
+      <c r="N20" t="str">
+        <v>1</v>
+      </c>
+      <c r="O20" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>Средство косметическое для ухода за волосами: маска для волос восстанавливающая с авокадо и маслом о</v>
-      </c>
-      <c r="B21">
-        <v>99000076210</v>
+        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея, 50 мл</v>
+      </c>
+      <c r="B21" t="str">
+        <v>99000176496</v>
       </c>
       <c r="C21" t="str">
-        <v>maska-batter_250ml</v>
-      </c>
-      <c r="D21">
-        <v>4670020497546</v>
-      </c>
-      <c r="E21">
-        <v>657</v>
-      </c>
-      <c r="F21">
-        <v>657</v>
-      </c>
-      <c r="G21">
-        <v>0</v>
-      </c>
-      <c r="H21">
-        <v>0</v>
-      </c>
-      <c r="I21">
-        <v>1</v>
-      </c>
-      <c r="J21">
-        <v>1</v>
-      </c>
-      <c r="K21">
-        <v>0</v>
-      </c>
-      <c r="L21">
-        <v>0</v>
-      </c>
-      <c r="M21">
-        <v>0</v>
-      </c>
-      <c r="N21">
-        <v>1</v>
-      </c>
-      <c r="O21">
-        <v>46230</v>
+        <v>retinait_krem_1_5_50</v>
+      </c>
+      <c r="D21" t="str">
+        <v>4660417421827</v>
+      </c>
+      <c r="E21" t="str">
+        <v>840</v>
+      </c>
+      <c r="F21" t="str">
+        <v>0</v>
+      </c>
+      <c r="G21" t="str">
+        <v>840</v>
+      </c>
+      <c r="H21" t="str">
+        <v>0</v>
+      </c>
+      <c r="I21" t="str">
+        <v>1</v>
+      </c>
+      <c r="J21" t="str">
+        <v>0</v>
+      </c>
+      <c r="K21" t="str">
+        <v>1</v>
+      </c>
+      <c r="L21" t="str">
+        <v>0</v>
+      </c>
+      <c r="M21" t="str">
+        <v>0</v>
+      </c>
+      <c r="N21" t="str">
+        <v>1</v>
+      </c>
+      <c r="O21" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Средство косметическое профессиональное: маска разогревающая для роста волос торговой марки: Алтея.</v>
-      </c>
-      <c r="B22">
-        <v>99000076208</v>
+        <v>Крем с липомосомальным ретинолом (0,1% - 3%), торговая марка Алтея</v>
+      </c>
+      <c r="B22" t="str">
+        <v>99000124418</v>
       </c>
       <c r="C22" t="str">
-        <v>maska-batter_dlya_ro</v>
-      </c>
-      <c r="D22">
-        <v>4603320465366</v>
-      </c>
-      <c r="E22">
-        <v>650</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-      <c r="G22">
-        <v>650</v>
-      </c>
-      <c r="H22">
-        <v>0</v>
-      </c>
-      <c r="I22">
-        <v>1</v>
-      </c>
-      <c r="J22">
-        <v>0</v>
-      </c>
-      <c r="K22">
-        <v>1</v>
-      </c>
-      <c r="L22">
-        <v>0</v>
-      </c>
-      <c r="M22">
-        <v>0</v>
-      </c>
-      <c r="N22">
-        <v>1</v>
-      </c>
-      <c r="O22">
-        <v>46230</v>
+        <v>retinait_krem_025_50</v>
+      </c>
+      <c r="D22" t="str">
+        <v>4660417421599</v>
+      </c>
+      <c r="E22" t="str">
+        <v>796</v>
+      </c>
+      <c r="F22" t="str">
+        <v>0</v>
+      </c>
+      <c r="G22" t="str">
+        <v>796</v>
+      </c>
+      <c r="H22" t="str">
+        <v>0</v>
+      </c>
+      <c r="I22" t="str">
+        <v>1</v>
+      </c>
+      <c r="J22" t="str">
+        <v>0</v>
+      </c>
+      <c r="K22" t="str">
+        <v>1</v>
+      </c>
+      <c r="L22" t="str">
+        <v>0</v>
+      </c>
+      <c r="M22" t="str">
+        <v>0</v>
+      </c>
+      <c r="N22" t="str">
+        <v>1</v>
+      </c>
+      <c r="O22" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Шампунь от перхоти лечебный с климбазолом Алтея, 250мл</v>
-      </c>
-      <c r="B23">
-        <v>99000076206</v>
+        <v>РЕТИНАЙТ сыворотка для лица 30 мл</v>
+      </c>
+      <c r="B23" t="str">
+        <v>99000125142</v>
       </c>
       <c r="C23" t="str">
-        <v>shampun_protiv_perho</v>
-      </c>
-      <c r="D23">
-        <v>4670020496679</v>
-      </c>
-      <c r="E23">
-        <v>650</v>
-      </c>
-      <c r="F23">
-        <v>0</v>
-      </c>
-      <c r="G23">
-        <v>650</v>
-      </c>
-      <c r="H23">
-        <v>0</v>
-      </c>
-      <c r="I23">
-        <v>1</v>
-      </c>
-      <c r="J23">
-        <v>0</v>
-      </c>
-      <c r="K23">
-        <v>1</v>
-      </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23">
-        <v>0</v>
-      </c>
-      <c r="N23">
-        <v>1</v>
-      </c>
-      <c r="O23">
-        <v>46230</v>
+        <v>retinait_syvorotka_1</v>
+      </c>
+      <c r="D23" t="str">
+        <v>4603320465403</v>
+      </c>
+      <c r="E23" t="str">
+        <v>780</v>
+      </c>
+      <c r="F23" t="str">
+        <v>0</v>
+      </c>
+      <c r="G23" t="str">
+        <v>780</v>
+      </c>
+      <c r="H23" t="str">
+        <v>0</v>
+      </c>
+      <c r="I23" t="str">
+        <v>1</v>
+      </c>
+      <c r="J23" t="str">
+        <v>0</v>
+      </c>
+      <c r="K23" t="str">
+        <v>1</v>
+      </c>
+      <c r="L23" t="str">
+        <v>0</v>
+      </c>
+      <c r="M23" t="str">
+        <v>0</v>
+      </c>
+      <c r="N23" t="str">
+        <v>1</v>
+      </c>
+      <c r="O23" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>Средство косметическое для ухода за волосами: масло для бороды, маркировка: Алтея.</v>
-      </c>
-      <c r="B24">
-        <v>99000076215</v>
+        <v>Крем для лица Ретинайт с церамидами, 50 мл</v>
+      </c>
+      <c r="B24" t="str">
+        <v>99000137436</v>
       </c>
       <c r="C24" t="str">
-        <v>maslo_dlya_borodi_50</v>
-      </c>
-      <c r="D24">
-        <v>4610172186882</v>
-      </c>
-      <c r="E24">
-        <v>569</v>
-      </c>
-      <c r="F24">
-        <v>0</v>
-      </c>
-      <c r="G24">
-        <v>569</v>
-      </c>
-      <c r="H24">
-        <v>0</v>
-      </c>
-      <c r="I24">
-        <v>1</v>
-      </c>
-      <c r="J24">
-        <v>0</v>
-      </c>
-      <c r="K24">
-        <v>1</v>
-      </c>
-      <c r="L24">
-        <v>0</v>
-      </c>
-      <c r="M24">
-        <v>0</v>
-      </c>
-      <c r="N24">
-        <v>1</v>
-      </c>
-      <c r="O24">
-        <v>46230</v>
+        <v>retinait_krem_01_50m</v>
+      </c>
+      <c r="D24" t="str">
+        <v>4660417421629</v>
+      </c>
+      <c r="E24" t="str">
+        <v>717</v>
+      </c>
+      <c r="F24" t="str">
+        <v>0</v>
+      </c>
+      <c r="G24" t="str">
+        <v>717</v>
+      </c>
+      <c r="H24" t="str">
+        <v>0</v>
+      </c>
+      <c r="I24" t="str">
+        <v>1</v>
+      </c>
+      <c r="J24" t="str">
+        <v>0</v>
+      </c>
+      <c r="K24" t="str">
+        <v>1</v>
+      </c>
+      <c r="L24" t="str">
+        <v>0</v>
+      </c>
+      <c r="M24" t="str">
+        <v>0</v>
+      </c>
+      <c r="N24" t="str">
+        <v>1</v>
+      </c>
+      <c r="O24" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
+        <v>Ретинайт 0,5 экспресс-омоложение Anti-Age Липосомальный комплекс ретинола 0,5 + Ниацинамид 50 мл</v>
+      </c>
+      <c r="B25" t="str">
+        <v>99000131675</v>
+      </c>
+      <c r="C25" t="str">
+        <v>retinait_krem_05_50m</v>
+      </c>
+      <c r="D25" t="str">
+        <v>4660417421759</v>
+      </c>
+      <c r="E25" t="str">
+        <v>702</v>
+      </c>
+      <c r="F25" t="str">
+        <v>0</v>
+      </c>
+      <c r="G25" t="str">
+        <v>702</v>
+      </c>
+      <c r="H25" t="str">
+        <v>0</v>
+      </c>
+      <c r="I25" t="str">
+        <v>1</v>
+      </c>
+      <c r="J25" t="str">
+        <v>0</v>
+      </c>
+      <c r="K25" t="str">
+        <v>1</v>
+      </c>
+      <c r="L25" t="str">
+        <v>0</v>
+      </c>
+      <c r="M25" t="str">
+        <v>0</v>
+      </c>
+      <c r="N25" t="str">
+        <v>1</v>
+      </c>
+      <c r="O25" t="str">
+        <v>28.7.2026</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
         <v>Шампунь для роста волос, от выпадения волос профессиональный, Алтея, 250 мл</v>
       </c>
-      <c r="B25">
+      <c r="B26" t="str">
         <v>99000076213</v>
       </c>
-      <c r="C25" t="str">
+      <c r="C26" t="str">
         <v>shampun_dlya_rosta_2</v>
       </c>
-      <c r="D25">
+      <c r="D26" t="str">
         <v>4670020496747</v>
       </c>
-      <c r="E25">
+      <c r="E26" t="str">
         <v>461</v>
       </c>
-      <c r="F25">
+      <c r="F26" t="str">
+        <v>0</v>
+      </c>
+      <c r="G26" t="str">
         <v>461</v>
       </c>
-      <c r="G25">
-        <v>0</v>
-      </c>
-      <c r="H25">
-        <v>0</v>
-      </c>
-      <c r="I25">
-        <v>1</v>
-      </c>
-      <c r="J25">
-        <v>1</v>
-      </c>
-      <c r="K25">
-        <v>0</v>
-      </c>
-      <c r="L25">
-        <v>0</v>
-      </c>
-      <c r="M25">
-        <v>0</v>
-      </c>
-      <c r="N25">
-        <v>1</v>
-      </c>
-      <c r="O25">
-        <v>46230</v>
+      <c r="H26" t="str">
+        <v>0</v>
+      </c>
+      <c r="I26" t="str">
+        <v>1</v>
+      </c>
+      <c r="J26" t="str">
+        <v>0</v>
+      </c>
+      <c r="K26" t="str">
+        <v>1</v>
+      </c>
+      <c r="L26" t="str">
+        <v>0</v>
+      </c>
+      <c r="M26" t="str">
+        <v>0</v>
+      </c>
+      <c r="N26" t="str">
+        <v>1</v>
+      </c>
+      <c r="O26" t="str">
+        <v>28.7.2026</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>Средство косметическое для ухода за волосами: масло для бороды, маркировка: Алтея.</v>
+      </c>
+      <c r="B27" t="str">
+        <v>99000076215</v>
+      </c>
+      <c r="C27" t="str">
+        <v>maslo_dlya_borodi_50</v>
+      </c>
+      <c r="D27" t="str">
+        <v>4610172186882</v>
+      </c>
+      <c r="E27" t="str">
+        <v>422</v>
+      </c>
+      <c r="F27" t="str">
+        <v>0</v>
+      </c>
+      <c r="G27" t="str">
+        <v>422</v>
+      </c>
+      <c r="H27" t="str">
+        <v>0</v>
+      </c>
+      <c r="I27" t="str">
+        <v>1</v>
+      </c>
+      <c r="J27" t="str">
+        <v>0</v>
+      </c>
+      <c r="K27" t="str">
+        <v>1</v>
+      </c>
+      <c r="L27" t="str">
+        <v>0</v>
+      </c>
+      <c r="M27" t="str">
+        <v>0</v>
+      </c>
+      <c r="N27" t="str">
+        <v>1</v>
+      </c>
+      <c r="O27" t="str">
+        <v>28.7.2026</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>Гель для интимной гигиены с молочной кислотой, Алтея, Интимвита, 300 мл</v>
+      </c>
+      <c r="B28" t="str">
+        <v>99000114723</v>
+      </c>
+      <c r="C28" t="str">
+        <v>intimvita_300ml</v>
+      </c>
+      <c r="D28" t="str">
+        <v>4630084865477</v>
+      </c>
+      <c r="E28" t="str">
+        <v>337</v>
+      </c>
+      <c r="F28" t="str">
+        <v>0</v>
+      </c>
+      <c r="G28" t="str">
+        <v>337</v>
+      </c>
+      <c r="H28" t="str">
+        <v>0</v>
+      </c>
+      <c r="I28" t="str">
+        <v>1</v>
+      </c>
+      <c r="J28" t="str">
+        <v>0</v>
+      </c>
+      <c r="K28" t="str">
+        <v>1</v>
+      </c>
+      <c r="L28" t="str">
+        <v>0</v>
+      </c>
+      <c r="M28" t="str">
+        <v>0</v>
+      </c>
+      <c r="N28" t="str">
+        <v>1</v>
+      </c>
+      <c r="O28" t="str">
+        <v>28.7.2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:O25"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O28"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:K6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -11850,15 +11991,15 @@
         <v>1</v>
       </c>
       <c r="K1" t="str">
-        <v>46230</v>
+        <v>28.07.2026</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>АЛТЕЯ-RETINT1</v>
+        <v>АЛТЕЯ-KRSPF50</v>
       </c>
       <c r="B2" t="str">
-        <v>Сыворотка с ретинолом 1% для лица от морщин антивозрастная Алтея 30 мл</v>
+        <v>Крем солнцезащитный СПФ 50 для лица 50 мл</v>
       </c>
       <c r="C2" t="str">
         <v>1</v>
@@ -11867,33 +12008,33 @@
         <v>0</v>
       </c>
       <c r="E2" t="str">
-        <v>660</v>
+        <v>701,5</v>
       </c>
       <c r="F2" t="str">
-        <v>143.82</v>
+        <v>132,6</v>
       </c>
       <c r="G2" t="str">
-        <v>429</v>
+        <v>455,98</v>
       </c>
       <c r="H2" t="str">
-        <v>231</v>
+        <v>245,52</v>
       </c>
       <c r="I2" t="str">
-        <v>retinait_syvorotka_1_30ml</v>
+        <v>krem_spf50_50ml</v>
       </c>
       <c r="J2" t="str">
         <v>1</v>
       </c>
       <c r="K2" t="str">
-        <v>46230</v>
+        <v>28.07.2026</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>АЛТЕЯ-KREMDLV</v>
+        <v>АЛТЕЯ-RETINT1</v>
       </c>
       <c r="B3" t="str">
-        <v>Крем для век и кожи вокруг глаз жидкие патчи для глаз Алтея 30 мл</v>
+        <v>Сыворотка с ретинолом 1% для лица от морщин антивозрастная Алтея 30 мл</v>
       </c>
       <c r="C3" t="str">
         <v>1</v>
@@ -11902,100 +12043,135 @@
         <v>0</v>
       </c>
       <c r="E3" t="str">
-        <v>547</v>
+        <v>660</v>
       </c>
       <c r="F3" t="str">
-        <v>126.5</v>
+        <v>143,82</v>
       </c>
       <c r="G3" t="str">
-        <v>355.55</v>
+        <v>429</v>
       </c>
       <c r="H3" t="str">
-        <v>191.45</v>
+        <v>231</v>
       </c>
       <c r="I3" t="str">
-        <v>krem_dlya_vek_30ml</v>
+        <v>retinait_syvorotka_1_30ml</v>
       </c>
       <c r="J3" t="str">
         <v>1</v>
       </c>
       <c r="K3" t="str">
-        <v>46230</v>
+        <v>28.07.2026</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>АЛТЕЯ-KREMRST</v>
+        <v>АЛТЕЯ-TERMSPR</v>
       </c>
       <c r="B4" t="str">
-        <v>Крем масло от растяжек для беременных и подростков с эластином Алтея 200 мл</v>
+        <v>Спрей для волос 17 в 1 восстанавливающий с кератином Алтея 200 мл</v>
       </c>
       <c r="C4" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D4" t="str">
         <v>0</v>
       </c>
       <c r="E4" t="str">
-        <v>710</v>
+        <v>326</v>
       </c>
       <c r="F4" t="str">
-        <v>302.4</v>
+        <v>116,1</v>
       </c>
       <c r="G4" t="str">
-        <v>511.2</v>
+        <v>234,72</v>
       </c>
       <c r="H4" t="str">
-        <v>198.8</v>
+        <v>91,28</v>
       </c>
       <c r="I4" t="str">
-        <v>krem_ot_rastyazhek</v>
+        <v>termo_sprei_200ml</v>
       </c>
       <c r="J4" t="str">
         <v>1</v>
       </c>
       <c r="K4" t="str">
-        <v>46230</v>
+        <v>28.07.2026</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>АЛТЕЯ-SHPPERH</v>
+        <v>АЛТЕЯ-KREMRST</v>
       </c>
       <c r="B5" t="str">
-        <v>Шампунь от перхоти лечебный с климбазолом Алтея 250 мл</v>
+        <v>Крем масло от растяжек для беременных и подростков с эластином Алтея 200 мл</v>
       </c>
       <c r="C5" t="str">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D5" t="str">
         <v>0</v>
       </c>
       <c r="E5" t="str">
-        <v>816.9</v>
+        <v>355</v>
       </c>
       <c r="F5" t="str">
-        <v>212.4</v>
+        <v>151,2</v>
       </c>
       <c r="G5" t="str">
-        <v>588.16</v>
+        <v>255,6</v>
       </c>
       <c r="H5" t="str">
-        <v>228.74</v>
+        <v>99,4</v>
       </c>
       <c r="I5" t="str">
-        <v>shampun_protiv_perhoti_250ml</v>
+        <v>krem_ot_rastyazhek</v>
       </c>
       <c r="J5" t="str">
         <v>1</v>
       </c>
       <c r="K5" t="str">
-        <v>46230</v>
+        <v>28.07.2026</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>АЛТЕЯ-REMYVRS</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Ремувер для снятия ресниц Алтея 18 г</v>
+      </c>
+      <c r="C6" t="str">
+        <v>1</v>
+      </c>
+      <c r="D6" t="str">
+        <v>0</v>
+      </c>
+      <c r="E6" t="str">
+        <v>341</v>
+      </c>
+      <c r="F6" t="str">
+        <v>80,92</v>
+      </c>
+      <c r="G6" t="str">
+        <v>245,52</v>
+      </c>
+      <c r="H6" t="str">
+        <v>95,48</v>
+      </c>
+      <c r="I6" t="str">
+        <v>nabor_remuver_kremovii</v>
+      </c>
+      <c r="J6" t="str">
+        <v>1</v>
+      </c>
+      <c r="K6" t="str">
+        <v>28.07.2026</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>